<commit_message>
feat: implement admin panel with secure API authentication and dynamic data management
</commit_message>
<xml_diff>
--- a/apps-script/DB-alazkar.xlsx
+++ b/apps-script/DB-alazkar.xlsx
@@ -432,7 +432,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>z7s9p2w8</v>
+        <v>zikir-setelah-shalat</v>
       </c>
       <c r="C2" t="str">
         <v>zikir_setelah_shalat</v>
@@ -447,7 +447,7 @@
         <v>lucide:book-marked</v>
       </c>
       <c r="G2" t="str">
-        <v>d3s7q1x5</v>
+        <v>doa-setelah-shalat</v>
       </c>
     </row>
     <row r="3">
@@ -455,7 +455,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>d3s7q1x5</v>
+        <v>doa-setelah-shalat</v>
       </c>
       <c r="C3" t="str">
         <v>doa_setelah_shalat</v>
@@ -478,7 +478,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>t9h2m6b4</v>
+        <v>tahlil</v>
       </c>
       <c r="C4" t="str">
         <v>tahlil</v>
@@ -493,7 +493,7 @@
         <v>lucide:book-open</v>
       </c>
       <c r="G4" t="str">
-        <v>d4t8k2y7</v>
+        <v>doa-tahlil</v>
       </c>
     </row>
     <row r="5">
@@ -501,7 +501,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>d4t8k2y7</v>
+        <v>doa-tahlil</v>
       </c>
       <c r="C5" t="str">
         <v>doa_tahlil</v>
@@ -524,7 +524,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>t5b7r9w2</v>
+        <v>takbiran</v>
       </c>
       <c r="C6" t="str">
         <v>takbiran</v>

</xml_diff>